<commit_message>
Update the Hardware Model of BLDC_FOC in Matlab 2025b, because the Matlab 2025b removed the Specific Power System. And add the motor model simulation scriptes in CodeSimulation/MotorSimScriptes
</commit_message>
<xml_diff>
--- a/BLDC_FOC/MotorControlData.xlsx
+++ b/BLDC_FOC/MotorControlData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\MotorControl\05_SystemSimulation\FloatPoint\FOC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UserProjects\MotorControlSim\MotorControllSimulation\BLDC_FOC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43E11C9-CBD3-4186-A923-20A7E9F6CE92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B736A542-F301-4F11-8C9F-9DF7D7B45D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1516,19 +1516,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L38"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.59765625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="9.1328125" style="2"/>
-    <col min="3" max="3" width="17.46484375" style="2" customWidth="1"/>
-    <col min="4" max="5" width="13.3984375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="12.46484375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="19.1328125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="30.3984375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="13.3984375" style="5" customWidth="1"/>
+    <col min="1" max="1" width="27.625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="9.125" style="2"/>
+    <col min="3" max="3" width="17.5" style="2" customWidth="1"/>
+    <col min="4" max="5" width="13.375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="12.5" style="2" customWidth="1"/>
+    <col min="7" max="7" width="19.125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="30.375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="13.375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" s="3" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1557,7 +1557,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
         <v>11</v>
       </c>
@@ -1586,7 +1586,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>133</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>134</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>13</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>15</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
         <v>72</v>
       </c>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="I7" s="12"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>71</v>
       </c>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="I8" s="12"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
         <v>34</v>
       </c>
@@ -1785,7 +1785,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>33</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
         <v>36</v>
       </c>
@@ -1844,7 +1844,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>42</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
         <v>43</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>44</v>
       </c>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="I14" s="12"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
         <v>45</v>
       </c>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="I15" s="12"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
         <v>31</v>
       </c>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="I16" s="12"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
         <v>38</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
         <v>39</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
         <v>40</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
         <v>187</v>
       </c>
@@ -2100,7 +2100,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
         <v>188</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>507.58718608572195</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
         <v>189</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
         <v>41</v>
       </c>
@@ -2193,7 +2193,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>55</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>56</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>57</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>58</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="12" t="s">
         <v>59</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="12" t="s">
         <v>182</v>
       </c>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="I29" s="12"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
         <v>183</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
         <v>184</v>
       </c>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="I31" s="12"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
         <v>185</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
         <v>70</v>
       </c>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="I33" s="12"/>
     </row>
-    <row r="34" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
         <v>138</v>
       </c>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="I34" s="12"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="12" t="s">
         <v>60</v>
       </c>
@@ -2534,7 +2534,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
         <v>139</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
         <v>61</v>
       </c>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="I37" s="12"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
         <v>62</v>
       </c>
@@ -2628,19 +2628,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58219796-439D-4218-8351-215451A32352}">
   <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.59765625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="9.1328125" style="2"/>
-    <col min="3" max="3" width="18.265625" style="2" customWidth="1"/>
-    <col min="4" max="5" width="13.3984375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="12.46484375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="19.1328125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="22.3984375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="13.3984375" style="5" customWidth="1"/>
+    <col min="1" max="1" width="21.625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="9.125" style="2"/>
+    <col min="3" max="3" width="18.25" style="2" customWidth="1"/>
+    <col min="4" max="5" width="13.375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="12.5" style="2" customWidth="1"/>
+    <col min="7" max="7" width="19.125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="22.375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="13.375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>22</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>23</v>
       </c>
@@ -2717,7 +2717,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>232</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>233</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>234</v>
       </c>
@@ -2819,19 +2819,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35A44938-6B5D-40C1-8F40-515C706BD968}">
   <dimension ref="A1:J63"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.265625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="15.73046875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="10.265625" style="4" customWidth="1"/>
-    <col min="4" max="5" width="13.3984375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="12.46484375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="19.1328125" style="4" customWidth="1"/>
-    <col min="8" max="8" width="13.3984375" style="4" customWidth="1"/>
-    <col min="9" max="9" width="13.3984375" style="7" customWidth="1"/>
+    <col min="1" max="1" width="28.25" style="4" customWidth="1"/>
+    <col min="2" max="2" width="15.75" style="4" customWidth="1"/>
+    <col min="3" max="3" width="10.25" style="4" customWidth="1"/>
+    <col min="4" max="5" width="13.375" style="4" customWidth="1"/>
+    <col min="6" max="6" width="12.5" style="4" customWidth="1"/>
+    <col min="7" max="7" width="19.125" style="4" customWidth="1"/>
+    <col min="8" max="8" width="13.375" style="4" customWidth="1"/>
+    <col min="9" max="9" width="13.375" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>105</v>
       </c>
@@ -2888,7 +2888,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>106</v>
       </c>
@@ -2914,7 +2914,7 @@
       </c>
       <c r="I3" s="19"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>159</v>
       </c>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="I4" s="19"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>186</v>
       </c>
@@ -2966,7 +2966,7 @@
       </c>
       <c r="I5" s="19"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>160</v>
       </c>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="I6" s="20"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>89</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>93</v>
       </c>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="I8" s="16"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>94</v>
       </c>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="I9" s="16"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>230</v>
       </c>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="I10" s="16"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
         <v>231</v>
       </c>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="I11" s="16"/>
     </row>
-    <row r="12" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>170</v>
       </c>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="I12" s="16"/>
     </row>
-    <row r="13" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>171</v>
       </c>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="I13" s="16"/>
     </row>
-    <row r="14" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>167</v>
       </c>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="I14" s="16"/>
     </row>
-    <row r="15" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
         <v>168</v>
       </c>
@@ -3230,7 +3230,7 @@
       </c>
       <c r="I15" s="17"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
         <v>91</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>97</v>
       </c>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="I17" s="19"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>98</v>
       </c>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="I18" s="19"/>
     </row>
-    <row r="19" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
         <v>108</v>
       </c>
@@ -3334,7 +3334,7 @@
       </c>
       <c r="I19" s="19"/>
     </row>
-    <row r="20" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
         <v>118</v>
       </c>
@@ -3359,7 +3359,7 @@
       </c>
       <c r="I20" s="19"/>
     </row>
-    <row r="21" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
         <v>111</v>
       </c>
@@ -3385,7 +3385,7 @@
       </c>
       <c r="I21" s="19"/>
     </row>
-    <row r="22" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
         <v>112</v>
       </c>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="I22" s="19"/>
     </row>
-    <row r="23" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>110</v>
       </c>
@@ -3437,7 +3437,7 @@
       </c>
       <c r="I23" s="19"/>
     </row>
-    <row r="24" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
         <v>113</v>
       </c>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="I24" s="19"/>
     </row>
-    <row r="25" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
         <v>119</v>
       </c>
@@ -3488,7 +3488,7 @@
       </c>
       <c r="I25" s="19"/>
     </row>
-    <row r="26" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
         <v>114</v>
       </c>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="I26" s="19"/>
     </row>
-    <row r="27" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
         <v>115</v>
       </c>
@@ -3540,7 +3540,7 @@
       </c>
       <c r="I27" s="19"/>
     </row>
-    <row r="28" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
         <v>116</v>
       </c>
@@ -3566,7 +3566,7 @@
       </c>
       <c r="I28" s="19"/>
     </row>
-    <row r="29" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A29" s="8" t="s">
         <v>117</v>
       </c>
@@ -3592,7 +3592,7 @@
       </c>
       <c r="I29" s="19"/>
     </row>
-    <row r="30" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
         <v>235</v>
       </c>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="I30" s="19"/>
     </row>
-    <row r="31" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>237</v>
       </c>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="I31" s="19"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
         <v>101</v>
       </c>
@@ -3674,7 +3674,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="9" t="s">
         <v>102</v>
       </c>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="I33" s="16"/>
     </row>
-    <row r="34" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A34" s="9" t="s">
         <v>155</v>
       </c>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="I34" s="16"/>
     </row>
-    <row r="35" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A35" s="10" t="s">
         <v>156</v>
       </c>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="I35" s="16"/>
     </row>
-    <row r="36" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A36" s="8" t="s">
         <v>165</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A37" s="8" t="s">
         <v>192</v>
       </c>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="I37" s="19"/>
     </row>
-    <row r="38" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A38" s="8" t="s">
         <v>193</v>
       </c>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="I38" s="19"/>
     </row>
-    <row r="39" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A39" s="8" t="s">
         <v>190</v>
       </c>
@@ -3855,7 +3855,7 @@
       </c>
       <c r="I39" s="19"/>
     </row>
-    <row r="40" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A40" s="8" t="s">
         <v>191</v>
       </c>
@@ -3881,7 +3881,7 @@
       </c>
       <c r="I40" s="20"/>
     </row>
-    <row r="41" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
         <v>200</v>
       </c>
@@ -3909,7 +3909,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A42" s="9" t="s">
         <v>199</v>
       </c>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="I42" s="16"/>
     </row>
-    <row r="43" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A43" s="9" t="s">
         <v>212</v>
       </c>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="I43" s="16"/>
     </row>
-    <row r="44" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A44" s="9" t="s">
         <v>213</v>
       </c>
@@ -3987,7 +3987,7 @@
       </c>
       <c r="I44" s="16"/>
     </row>
-    <row r="45" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A45" s="9" t="s">
         <v>201</v>
       </c>
@@ -4017,7 +4017,7 @@
         <v>507.58718608572195</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A46" s="9" t="s">
         <v>202</v>
       </c>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="I46" s="16"/>
     </row>
-    <row r="47" spans="1:10" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A47" s="9" t="s">
         <v>211</v>
       </c>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="I47" s="16"/>
     </row>
-    <row r="48" spans="1:10" ht="41.65" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:10" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A48" s="9" t="s">
         <v>214</v>
       </c>
@@ -4093,7 +4093,7 @@
       </c>
       <c r="I48" s="17"/>
     </row>
-    <row r="49" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A49" s="8" t="s">
         <v>107</v>
       </c>
@@ -4120,7 +4120,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A50" s="8" t="s">
         <v>103</v>
       </c>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="I50" s="19"/>
     </row>
-    <row r="51" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A51" s="8" t="s">
         <v>104</v>
       </c>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="I51" s="19"/>
     </row>
-    <row r="52" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A52" s="8" t="s">
         <v>217</v>
       </c>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="I52" s="19"/>
     </row>
-    <row r="53" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A53" s="8" t="s">
         <v>215</v>
       </c>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="I53" s="19"/>
     </row>
-    <row r="54" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A54" s="8" t="s">
         <v>216</v>
       </c>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="I54" s="19"/>
     </row>
-    <row r="55" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A55" s="8" t="s">
         <v>224</v>
       </c>
@@ -4274,7 +4274,7 @@
       </c>
       <c r="I55" s="19"/>
     </row>
-    <row r="56" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A56" s="8" t="s">
         <v>225</v>
       </c>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="I56" s="19"/>
     </row>
-    <row r="57" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A57" s="8" t="s">
         <v>226</v>
       </c>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="I57" s="20"/>
     </row>
-    <row r="58" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A58" s="9" t="s">
         <v>85</v>
       </c>
@@ -4353,7 +4353,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
         <v>87</v>
       </c>
@@ -4378,7 +4378,7 @@
       </c>
       <c r="I59" s="16"/>
     </row>
-    <row r="60" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A60" s="9" t="s">
         <v>176</v>
       </c>
@@ -4404,7 +4404,7 @@
       </c>
       <c r="I60" s="16"/>
     </row>
-    <row r="61" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A61" s="9" t="s">
         <v>142</v>
       </c>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="I61" s="16"/>
     </row>
-    <row r="62" spans="1:9" ht="27.75" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A62" s="9" t="s">
         <v>144</v>
       </c>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="I62" s="17"/>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C63" s="4" t="s">
         <v>177</v>
       </c>
@@ -4479,20 +4479,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FBE0796-AE15-466F-8ACC-98F71496990C}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.59765625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="9.1328125" style="2"/>
+    <col min="1" max="1" width="13.625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="9.125" style="2"/>
     <col min="3" max="3" width="13" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.265625" style="2" customWidth="1"/>
-    <col min="5" max="6" width="13.3984375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="12.46484375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="19.1328125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="12.265625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="13.3984375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.25" style="2" customWidth="1"/>
+    <col min="5" max="6" width="13.375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12.5" style="2" customWidth="1"/>
+    <col min="8" max="8" width="19.125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="12.25" style="2" customWidth="1"/>
+    <col min="10" max="10" width="13.375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4524,7 +4524,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -4565,12 +4565,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85608A1-FBFE-45A4-A499-4015C1D010B6}">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.265625" customWidth="1"/>
+    <col min="2" max="2" width="11.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -4593,7 +4593,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1454F5CE-E61B-48C8-A153-EE4DC3929049}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4603,7 +4603,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{145BA5FC-E68D-46C0-B305-755132DD04FD}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>